<commit_message>
Complete PMIP market growth intelligence analysis
</commit_message>
<xml_diff>
--- a/PMIP_Gantt_Chart.xlsx
+++ b/PMIP_Gantt_Chart.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/richardakole/Documents/Final-year-projects/PMIP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/richardakole/Documents/Now/PMIP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD82A15-A591-C44E-A2DF-3676C6074B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E362AEB8-C575-8E4B-A202-773FDF2F7CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15100" yWindow="660" windowWidth="15140" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -839,7 +839,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -882,7 +882,7 @@
       <c r="AB1" s="22"/>
       <c r="AC1" s="22"/>
     </row>
-    <row r="3" spans="1:29" ht="15">
+    <row r="3" spans="1:29">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -910,7 +910,7 @@
       <c r="L3" s="23"/>
       <c r="M3" s="23"/>
     </row>
-    <row r="4" spans="1:29" ht="15">
+    <row r="4" spans="1:29">
       <c r="A4" s="2">
         <v>46258</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>46412</v>
       </c>
     </row>
-    <row r="8" spans="1:29" ht="31">
+    <row r="8" spans="1:29" ht="32">
       <c r="A8" s="13" t="s">
         <v>15</v>
       </c>
@@ -1077,7 +1077,7 @@
       <c r="AB8" s="5"/>
       <c r="AC8" s="10"/>
     </row>
-    <row r="9" spans="1:29" ht="16">
+    <row r="9" spans="1:29" ht="32">
       <c r="A9" s="13" t="s">
         <v>17</v>
       </c>
@@ -1122,7 +1122,7 @@
       <c r="AB9" s="5"/>
       <c r="AC9" s="10"/>
     </row>
-    <row r="10" spans="1:29" ht="31">
+    <row r="10" spans="1:29" ht="32">
       <c r="A10" s="13" t="s">
         <v>19</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>4</v>
       </c>
       <c r="F12" s="16">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G12" s="5">
         <v>1</v>
@@ -1257,7 +1257,7 @@
       <c r="AB12" s="5"/>
       <c r="AC12" s="10"/>
     </row>
-    <row r="13" spans="1:29" ht="15">
+    <row r="13" spans="1:29" ht="16">
       <c r="A13" s="13" t="s">
         <v>23</v>
       </c>
@@ -1271,10 +1271,7 @@
         <v>46268</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G13" s="5">
         <v>1</v>
@@ -1304,7 +1301,7 @@
       <c r="AB13" s="5"/>
       <c r="AC13" s="10"/>
     </row>
-    <row r="14" spans="1:29" ht="15">
+    <row r="14" spans="1:29" ht="16">
       <c r="A14" s="13" t="s">
         <v>23</v>
       </c>
@@ -1318,7 +1315,7 @@
         <v>46275</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F14" s="16">
         <v>0</v>
@@ -1351,7 +1348,7 @@
       <c r="AB14" s="5"/>
       <c r="AC14" s="10"/>
     </row>
-    <row r="15" spans="1:29" ht="15">
+    <row r="15" spans="1:29" ht="16">
       <c r="A15" s="13" t="s">
         <v>27</v>
       </c>
@@ -1365,7 +1362,7 @@
         <v>46278</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F15" s="16">
         <v>0</v>
@@ -1396,7 +1393,7 @@
       <c r="AB15" s="5"/>
       <c r="AC15" s="10"/>
     </row>
-    <row r="16" spans="1:29" ht="30">
+    <row r="16" spans="1:29" ht="32">
       <c r="A16" s="13" t="s">
         <v>29</v>
       </c>
@@ -1410,7 +1407,7 @@
         <v>46287</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F16" s="16">
         <v>0</v>
@@ -1445,7 +1442,7 @@
       <c r="AB16" s="5"/>
       <c r="AC16" s="10"/>
     </row>
-    <row r="17" spans="1:29" ht="15">
+    <row r="17" spans="1:29" ht="16">
       <c r="A17" s="13" t="s">
         <v>29</v>
       </c>
@@ -1459,7 +1456,7 @@
         <v>46294</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F17" s="16">
         <v>0</v>
@@ -1494,7 +1491,7 @@
       <c r="AB17" s="5"/>
       <c r="AC17" s="10"/>
     </row>
-    <row r="18" spans="1:29" ht="30">
+    <row r="18" spans="1:29" ht="32">
       <c r="A18" s="13" t="s">
         <v>32</v>
       </c>
@@ -1508,7 +1505,7 @@
         <v>46304</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F18" s="16">
         <v>0</v>
@@ -1541,7 +1538,7 @@
       <c r="AB18" s="5"/>
       <c r="AC18" s="10"/>
     </row>
-    <row r="19" spans="1:29" ht="15">
+    <row r="19" spans="1:29" ht="32">
       <c r="A19" s="13" t="s">
         <v>34</v>
       </c>
@@ -1555,7 +1552,7 @@
         <v>46313</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F19" s="16">
         <v>0</v>
@@ -1588,7 +1585,7 @@
       <c r="AB19" s="5"/>
       <c r="AC19" s="10"/>
     </row>
-    <row r="20" spans="1:29" ht="15">
+    <row r="20" spans="1:29" ht="16">
       <c r="A20" s="13" t="s">
         <v>36</v>
       </c>
@@ -1635,7 +1632,7 @@
       <c r="AB20" s="5"/>
       <c r="AC20" s="10"/>
     </row>
-    <row r="21" spans="1:29" ht="15">
+    <row r="21" spans="1:29" ht="16">
       <c r="A21" s="13" t="s">
         <v>38</v>
       </c>
@@ -1682,7 +1679,7 @@
       <c r="AB21" s="5"/>
       <c r="AC21" s="10"/>
     </row>
-    <row r="22" spans="1:29" ht="15">
+    <row r="22" spans="1:29" ht="16">
       <c r="A22" s="13" t="s">
         <v>40</v>
       </c>
@@ -1729,7 +1726,7 @@
       <c r="AB22" s="5"/>
       <c r="AC22" s="10"/>
     </row>
-    <row r="23" spans="1:29" ht="15">
+    <row r="23" spans="1:29" ht="16">
       <c r="A23" s="13" t="s">
         <v>42</v>
       </c>
@@ -1776,7 +1773,7 @@
       <c r="AB23" s="5"/>
       <c r="AC23" s="10"/>
     </row>
-    <row r="24" spans="1:29" ht="15">
+    <row r="24" spans="1:29" ht="16">
       <c r="A24" s="13" t="s">
         <v>44</v>
       </c>
@@ -1823,7 +1820,7 @@
       <c r="AB24" s="5"/>
       <c r="AC24" s="10"/>
     </row>
-    <row r="25" spans="1:29" ht="15">
+    <row r="25" spans="1:29" ht="16">
       <c r="A25" s="13" t="s">
         <v>46</v>
       </c>
@@ -1870,7 +1867,7 @@
       <c r="AB25" s="5"/>
       <c r="AC25" s="10"/>
     </row>
-    <row r="26" spans="1:29" ht="15">
+    <row r="26" spans="1:29" ht="16">
       <c r="A26" s="13" t="s">
         <v>48</v>
       </c>
@@ -1917,7 +1914,7 @@
       <c r="AB26" s="5"/>
       <c r="AC26" s="10"/>
     </row>
-    <row r="27" spans="1:29" ht="30">
+    <row r="27" spans="1:29" ht="32">
       <c r="A27" s="13" t="s">
         <v>50</v>
       </c>
@@ -1966,7 +1963,7 @@
       <c r="AB27" s="5"/>
       <c r="AC27" s="10"/>
     </row>
-    <row r="28" spans="1:29" ht="15">
+    <row r="28" spans="1:29" ht="16">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
@@ -2015,7 +2012,7 @@
       <c r="AB28" s="5"/>
       <c r="AC28" s="10"/>
     </row>
-    <row r="29" spans="1:29" ht="15">
+    <row r="29" spans="1:29" ht="16">
       <c r="A29" s="13" t="s">
         <v>54</v>
       </c>
@@ -2064,7 +2061,7 @@
       <c r="AB29" s="5"/>
       <c r="AC29" s="10"/>
     </row>
-    <row r="30" spans="1:29" ht="15">
+    <row r="30" spans="1:29" ht="16">
       <c r="A30" s="13" t="s">
         <v>56</v>
       </c>
@@ -2113,7 +2110,7 @@
       <c r="AB30" s="5"/>
       <c r="AC30" s="10"/>
     </row>
-    <row r="31" spans="1:29" ht="15">
+    <row r="31" spans="1:29" ht="32">
       <c r="A31" s="13" t="s">
         <v>58</v>
       </c>
@@ -2162,7 +2159,7 @@
       </c>
       <c r="AC31" s="10"/>
     </row>
-    <row r="32" spans="1:29" ht="15">
+    <row r="32" spans="1:29" ht="16">
       <c r="A32" s="13" t="s">
         <v>60</v>
       </c>
@@ -2209,7 +2206,7 @@
       </c>
       <c r="AC32" s="10"/>
     </row>
-    <row r="33" spans="1:29" ht="30">
+    <row r="33" spans="1:29" ht="32">
       <c r="A33" s="17" t="s">
         <v>62</v>
       </c>
@@ -2280,7 +2277,7 @@
       <formula>E8="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F8:F33">
+  <conditionalFormatting sqref="F14:F33 F8:F12">
     <cfRule type="dataBar" priority="9">
       <dataBar>
         <cfvo type="min"/>
@@ -2333,7 +2330,7 @@
               <x14:axisColor auto="1"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>F8:F33</xm:sqref>
+          <xm:sqref>F14:F33 F8:F12</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -2344,7 +2341,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>

</xml_diff>